<commit_message>
Progress on autoblocked tabs page
Automated migration updates generated by Experience Modernization Agent.

Changed files (9):
- scripts/scripts.js
- scripts/section-tabs.js
- styles/styles.css
- tools/importer/import-reports-and-presentations.bundle.js
- tools/importer/import-reports-and-presentations.js
- tools/importer/parsers/cards-feature-reports.js
- tools/importer/reports/en/investors/reports-and-presentations.report.json
- tools/importer/reports/import-reports-and-presentations.report.xlsx
- tools/importer/transformers/atlascopcogroup-reports-tabs.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-reports-and-presentations.report.xlsx
+++ b/tools/importer/reports/import-reports-and-presentations.report.xlsx
@@ -64,7 +64,7 @@
     <t>en/investors/reports-and-presentations.report.json</t>
   </si>
   <si>
-    <t>[]</t>
+    <t>["cards-feature"]</t>
   </si>
   <si>
     <t>en/investors/reports-and-presentations</t>
@@ -73,7 +73,7 @@
     <t>reports-and-presentations</t>
   </si>
   <si>
-    <t>2026-08-10T15:15:28.239Z</t>
+    <t>2026-08-10T16:24:17.541Z</t>
   </si>
   <si>
     <t>Reports and presentations</t>

</xml_diff>